<commit_message>
knited version - calc of reliability
</commit_message>
<xml_diff>
--- a/Reproduce6 - AnalysisBySystem/Data_Analysis/generatedData/EFA_Summary_Consolidated.xlsx
+++ b/Reproduce6 - AnalysisBySystem/Data_Analysis/generatedData/EFA_Summary_Consolidated.xlsx
@@ -596,25 +596,25 @@
         <v>5.41</v>
       </c>
       <c r="G2" t="n">
-        <v>0.755</v>
+        <v>0.791</v>
       </c>
       <c r="H2" t="n">
         <v>0.888</v>
       </c>
       <c r="I2" t="n">
-        <v>0.363</v>
+        <v>0.38</v>
       </c>
       <c r="J2" t="n">
         <v>0.533</v>
       </c>
       <c r="K2" t="n">
-        <v>0.275</v>
+        <v>0.28</v>
       </c>
       <c r="L2" t="n">
         <v>0.283</v>
       </c>
       <c r="M2" t="n">
-        <v>0.201</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="3">
@@ -637,25 +637,25 @@
         <v>4.609</v>
       </c>
       <c r="G3" t="n">
-        <v>1.244</v>
+        <v>1.248</v>
       </c>
       <c r="H3" t="n">
         <v>1.194</v>
       </c>
       <c r="I3" t="n">
-        <v>0.806</v>
+        <v>0.799</v>
       </c>
       <c r="J3" t="n">
         <v>0.721</v>
       </c>
       <c r="K3" t="n">
-        <v>0.592</v>
+        <v>0.595</v>
       </c>
       <c r="L3" t="n">
         <v>0.46</v>
       </c>
       <c r="M3" t="n">
-        <v>0.41</v>
+        <v>0.424</v>
       </c>
     </row>
     <row r="4">
@@ -678,25 +678,25 @@
         <v>6.006</v>
       </c>
       <c r="G4" t="n">
-        <v>1.327</v>
+        <v>1.322</v>
       </c>
       <c r="H4" t="n">
         <v>1.267</v>
       </c>
       <c r="I4" t="n">
-        <v>0.828</v>
+        <v>0.831</v>
       </c>
       <c r="J4" t="n">
         <v>0.808</v>
       </c>
       <c r="K4" t="n">
-        <v>0.621</v>
+        <v>0.628</v>
       </c>
       <c r="L4" t="n">
         <v>0.334</v>
       </c>
       <c r="M4" t="n">
-        <v>0.443</v>
+        <v>0.441</v>
       </c>
     </row>
     <row r="5">
@@ -719,25 +719,25 @@
         <v>5.935</v>
       </c>
       <c r="G5" t="n">
-        <v>1.48</v>
+        <v>1.465</v>
       </c>
       <c r="H5" t="n">
         <v>0.785</v>
       </c>
       <c r="I5" t="n">
-        <v>0.921</v>
+        <v>0.936</v>
       </c>
       <c r="J5" t="n">
         <v>0.73</v>
       </c>
       <c r="K5" t="n">
-        <v>0.687</v>
+        <v>0.685</v>
       </c>
       <c r="L5" t="n">
         <v>0.418</v>
       </c>
       <c r="M5" t="n">
-        <v>0.479</v>
+        <v>0.465</v>
       </c>
     </row>
     <row r="6">
@@ -760,25 +760,25 @@
         <v>6.396</v>
       </c>
       <c r="G6" t="n">
-        <v>1.263</v>
+        <v>1.277</v>
       </c>
       <c r="H6" t="n">
         <v>1.442</v>
       </c>
       <c r="I6" t="n">
-        <v>0.824</v>
+        <v>0.825</v>
       </c>
       <c r="J6" t="n">
         <v>0.363</v>
       </c>
       <c r="K6" t="n">
-        <v>0.612</v>
+        <v>0.614</v>
       </c>
       <c r="L6" t="n">
         <v>0.346</v>
       </c>
       <c r="M6" t="n">
-        <v>0.439</v>
+        <v>0.432</v>
       </c>
     </row>
     <row r="7">
@@ -807,7 +807,7 @@
         <v>1.02</v>
       </c>
       <c r="I7" t="n">
-        <v>0.829</v>
+        <v>0.811</v>
       </c>
       <c r="J7" t="n">
         <v>0.806</v>
@@ -819,7 +819,7 @@
         <v>0.308</v>
       </c>
       <c r="M7" t="n">
-        <v>0.431</v>
+        <v>0.434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>